<commit_message>
Add the neighbouring Kycon series and the KPJX drilling plan
The catalogue photo of the wanted part cannot by itself separate KPJX
from the visually similar KPJ series, nor shielded from unshielded, so
both KPJ variants and the high-temperature KPJXHT are now listed
alongside the KPJX rows, each with the product URL exactly as search
returned it plus a token-free search fallback.

The measurements sheet now carries the manufacturer drilling plan so the
footprint can be compared hole by hole, which is what actually settles
the choice.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ge7EoEedmTKdVGHi238WWF
</commit_message>
<xml_diff>
--- a/exports/Liste-Mouser-Tonwelt-TG288.xlsx
+++ b/exports/Liste-Mouser-Tonwelt-TG288.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Sources &amp; statuts" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Liste Mouser'!$A$4:$G$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Liste Mouser'!$A$4:$G$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -524,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -689,12 +689,12 @@
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>Fiche mâle d'accouplement (réfection du cordon)</t>
+          <t>Prise alimentation DIN puissance 4 contacts — série voisine KPJ, non blindée</t>
         </is>
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>KPPX-4P</t>
+          <t>KPJ-4S</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
@@ -704,332 +704,332 @@
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>Variante</t>
+          <t>À départager</t>
         </is>
       </c>
       <c r="E8" s="7" t="n"/>
       <c r="F8" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/ProductDetail/Kycon/KPPX-4P?qs=Y0vc5luVLxJNKFay3ZyJLw%3D%3D</t>
+          <t>https://www.mouser.com/ProductDetail/Kycon/KPJ-4S?qs=/XicOQBKAMa%252BcJ0hGGZaig%3D%3D</t>
         </is>
       </c>
       <c r="G8" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=KPPX-4P</t>
+          <t>https://www.mouser.fr/c/?q=KPJ-4S</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Prise jack 3,5 mm, traversante</t>
+          <t>Prise alimentation DIN puissance 4 contacts — série voisine KPJ, blindée</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>SJ-43514</t>
+          <t>KPJ-4S-S</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Same Sky (CUI Devices)</t>
+          <t>Kycon</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Documenté</t>
+          <t>À départager</t>
         </is>
       </c>
       <c r="E9" s="7" t="n"/>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/ProductDetail/Same-Sky/SJ-43514?qs=WyjlAZoYn51bsBOfuwwiuw%3D%3D</t>
+          <t>https://www.mouser.com/ProductDetail/Kycon/KPJ-4S-S?qs=SrUfdAPSdgAPLkBk%2BStEGA%3D%3D</t>
         </is>
       </c>
       <c r="G9" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=SJ-43514</t>
+          <t>https://www.mouser.fr/c/?q=KPJ-4S-S</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>Prise jack 3,5 mm, CMS</t>
+          <t>Prise alimentation DIN puissance 4 contacts — version haute température</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>SJ-43514-SMT-TR</t>
+          <t>KPJXHT-4S-S</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>Same Sky (CUI Devices)</t>
+          <t>Kycon</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
         <is>
-          <t>Documenté</t>
+          <t>Variante</t>
         </is>
       </c>
       <c r="E10" s="7" t="n"/>
       <c r="F10" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/ProductDetail/CUI-Devices/SJ-43514-SMT-TR/?qs=WyjlAZoYn528%252BiAb5RzVtg%3D%3D</t>
+          <t>https://www.mouser.com/ProductDetail/Kycon/KPJXHT-4S-S?qs=6olcXJbp99TwdwXWG%2BzyAQ%3D%3D</t>
         </is>
       </c>
       <c r="G10" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=SJ-43514-SMT-TR</t>
+          <t>https://www.mouser.fr/c/?q=KPJXHT-4S-S</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Micro-USB B, CMS coudée</t>
+          <t>Fiche mâle d'accouplement (réfection du cordon)</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>10118193-0001LF</t>
+          <t>KPPX-4P</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Amphenol FCI</t>
+          <t>Kycon</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Documenté</t>
+          <t>Variante</t>
         </is>
       </c>
       <c r="E11" s="7" t="n"/>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/ProductDetail/Amphenol-FCI/10118193-0001LF?qs=Ywefl8B65e63Nsqd%2B8HZaQ%3D%3D</t>
+          <t>https://www.mouser.com/ProductDetail/Kycon/KPPX-4P?qs=Y0vc5luVLxJNKFay3ZyJLw%3D%3D</t>
         </is>
       </c>
       <c r="G11" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=10118193-0001LF</t>
+          <t>https://www.mouser.fr/c/?q=KPPX-4P</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>Micro-USB B, variante de montage</t>
+          <t>Prise jack 3,5 mm, traversante</t>
         </is>
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>10118192-0001LF</t>
+          <t>SJ-43514</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Amphenol FCI</t>
+          <t>Same Sky (CUI Devices)</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Variante</t>
+          <t>Documenté</t>
         </is>
       </c>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/ProductDetail/Amphenol-FCI/10118192-0001LF?qs=Ywefl8B65e5bHFoQtIudZg%3D%3D</t>
+          <t>https://www.mouser.com/ProductDetail/Same-Sky/SJ-43514?qs=WyjlAZoYn51bsBOfuwwiuw%3D%3D</t>
         </is>
       </c>
       <c r="G12" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=10118192-0001LF</t>
+          <t>https://www.mouser.fr/c/?q=SJ-43514</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Micro-USB B, variante de montage</t>
+          <t>Prise jack 3,5 mm, CMS</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>10118194-0001LF</t>
+          <t>SJ-43514-SMT-TR</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Amphenol FCI</t>
+          <t>Same Sky (CUI Devices)</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Variante</t>
+          <t>Documenté</t>
         </is>
       </c>
       <c r="E13" s="7" t="n"/>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/en/ProductDetail/Amphenol-FCI/10118194-0001LF?qs=Ywefl8B65e4FIdY8OWfRQA%3D%3D</t>
+          <t>https://www.mouser.com/ProductDetail/CUI-Devices/SJ-43514-SMT-TR/?qs=WyjlAZoYn528%252BiAb5RzVtg%3D%3D</t>
         </is>
       </c>
       <c r="G13" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=10118194-0001LF</t>
+          <t>https://www.mouser.fr/c/?q=SJ-43514-SMT-TR</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>Mini-USB B, 5 contacts</t>
+          <t>Micro-USB B, CMS coudée</t>
         </is>
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>54819-0519</t>
+          <t>10118193-0001LF</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Molex</t>
+          <t>Amphenol FCI</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>À confirmer</t>
+          <t>Documenté</t>
         </is>
       </c>
       <c r="E14" s="7" t="n"/>
       <c r="F14" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/ProductDetail/Molex/54819-0519?qs=x6EjVpvqMVObi%2BAAyuuEww%3D%3D</t>
+          <t>https://www.mouser.com/ProductDetail/Amphenol-FCI/10118193-0001LF?qs=Ywefl8B65e63Nsqd%2B8HZaQ%3D%3D</t>
         </is>
       </c>
       <c r="G14" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=54819-0519</t>
+          <t>https://www.mouser.fr/c/?q=10118193-0001LF</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>USB-C, 16 contacts, traversante</t>
+          <t>Micro-USB B, variante de montage</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>USB4085-GF-A</t>
+          <t>10118192-0001LF</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>GCT</t>
+          <t>Amphenol FCI</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>À confirmer</t>
+          <t>Variante</t>
         </is>
       </c>
       <c r="E15" s="7" t="n"/>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/ProductDetail/GCT/USB4085-GF-A?qs=KUoIvG%2F9Ilba1bQOahfWjw%3D%3D</t>
+          <t>https://www.mouser.com/ProductDetail/Amphenol-FCI/10118192-0001LF?qs=Ywefl8B65e5bHFoQtIudZg%3D%3D</t>
         </is>
       </c>
       <c r="G15" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=USB4085-GF-A</t>
+          <t>https://www.mouser.fr/c/?q=10118192-0001LF</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>Fusible réarmable PPTC, boîtier 1812</t>
+          <t>Micro-USB B, variante de montage</t>
         </is>
       </c>
       <c r="B16" s="10" t="inlineStr">
         <is>
-          <t>série MF-MSMF</t>
+          <t>10118194-0001LF</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>Bourns</t>
+          <t>Amphenol FCI</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>À confirmer</t>
+          <t>Variante</t>
         </is>
       </c>
       <c r="E16" s="7" t="n"/>
       <c r="F16" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/new/bourns/bourns-mf-msmf-series-fuses/</t>
+          <t>https://www.mouser.com/en/ProductDetail/Amphenol-FCI/10118194-0001LF?qs=Ywefl8B65e4FIdY8OWfRQA%3D%3D</t>
         </is>
       </c>
       <c r="G16" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=MF-MSMF</t>
+          <t>https://www.mouser.fr/c/?q=10118194-0001LF</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Fusibles PPTC — catalogue complet</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>Mini-USB B, 5 contacts</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>54819-0519</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Molex</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>Catalogue</t>
+          <t>À confirmer</t>
         </is>
       </c>
       <c r="E17" s="7" t="n"/>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/c/circuit-protection/thermistors/resettable-fuses-pptc/</t>
+          <t>https://www.mouser.com/ProductDetail/Molex/54819-0519?qs=x6EjVpvqMVObi%2BAAyuuEww%3D%3D</t>
         </is>
       </c>
       <c r="G17" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=fusible+PPTC+1812</t>
+          <t>https://www.mouser.fr/c/?q=54819-0519</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>Haut-parleur Ø15 mm, 8 Ω</t>
+          <t>USB-C, 16 contacts, traversante</t>
         </is>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
-          <t>AS01508MR-6-R</t>
+          <t>USB4085-GF-A</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>PUI Audio</t>
+          <t>GCT</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
@@ -1040,95 +1040,95 @@
       <c r="E18" s="7" t="n"/>
       <c r="F18" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/ProductDetail/PUI-Audio/AS01508MR-6-R?qs=vgjKjNJexThgIp5KgUGpgA%3D%3D</t>
+          <t>https://www.mouser.com/ProductDetail/GCT/USB4085-GF-A?qs=KUoIvG%2F9Ilba1bQOahfWjw%3D%3D</t>
         </is>
       </c>
       <c r="G18" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=AS01508MR-6-R</t>
+          <t>https://www.mouser.fr/c/?q=USB4085-GF-A</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Haut-parleurs — catalogue</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>Fusible réarmable PPTC, boîtier 1812</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>série MF-MSMF</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Bourns</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Catalogue</t>
+          <t>À confirmer</t>
         </is>
       </c>
       <c r="E19" s="7" t="n"/>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/en/c/electromechanical/audio-devices/speakers-transducers/</t>
+          <t>https://www.mouser.com/new/bourns/bourns-mf-msmf-series-fuses/</t>
         </is>
       </c>
       <c r="G19" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=haut-parleur+15mm+8+ohm</t>
+          <t>https://www.mouser.fr/c/?q=MF-MSMF</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>Bouton poussoir CMS (ceux de la carte)</t>
-        </is>
-      </c>
-      <c r="B20" s="10" t="inlineStr">
-        <is>
-          <t>SKRPACE010</t>
+          <t>Fusibles PPTC — catalogue complet</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>Alps Alpine</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Vu</t>
+          <t>Catalogue</t>
         </is>
       </c>
       <c r="E20" s="7" t="n"/>
       <c r="F20" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/ProductDetail/Alps-Alpine/SKRPACE010?qs=dHDuPHwQO79W8iY66hDbLQ%3D%3D</t>
+          <t>https://www.mouser.com/c/circuit-protection/thermistors/resettable-fuses-pptc/</t>
         </is>
       </c>
       <c r="G20" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=SKRPACE010</t>
+          <t>https://www.mouser.fr/c/?q=fusible+PPTC+1812</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Bouton poussoir traversant 6 × 6 mm</t>
+          <t>Haut-parleur Ø15 mm, 8 Ω</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>B3F-1000</t>
+          <t>AS01508MR-6-R</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Omron</t>
+          <t>PUI Audio</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -1139,217 +1139,217 @@
       <c r="E21" s="7" t="n"/>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/ProductDetail/Omron-Electronics/B3F-1000?qs=lK7M36XCk6JQHckSc1xIsg%3D%3D</t>
+          <t>https://www.mouser.com/ProductDetail/PUI-Audio/AS01508MR-6-R?qs=vgjKjNJexThgIp5KgUGpgA%3D%3D</t>
         </is>
       </c>
       <c r="G21" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=B3F-1000</t>
+          <t>https://www.mouser.fr/c/?q=AS01508MR-6-R</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>Antenne UHF hélicoïdale CMS</t>
-        </is>
-      </c>
-      <c r="B22" s="10" t="inlineStr">
-        <is>
-          <t>ANT-868-VHETH</t>
+          <t>Haut-parleurs — catalogue</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>TE / Linx</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D22" s="11" t="inlineStr">
         <is>
-          <t>Documenté</t>
+          <t>Catalogue</t>
         </is>
       </c>
       <c r="E22" s="7" t="n"/>
       <c r="F22" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/ProductDetail/TE-Connectivity-Linx-Technologies/ANT-868-VHETH?qs=pUKx8fyJudBCulCrBA9DxA%3D%3D</t>
+          <t>https://www.mouser.com/en/c/electromechanical/audio-devices/speakers-transducers/</t>
         </is>
       </c>
       <c r="G22" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=ANT-868-VHETH</t>
+          <t>https://www.mouser.fr/c/?q=haut-parleur+15mm+8+ohm</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Antenne UHF monopole embarqué Ø7 mm</t>
+          <t>Bouton poussoir CMS (ceux de la carte)</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>ANT-868-JJB-ST</t>
+          <t>SKRPACE010</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>TE / Linx</t>
+          <t>Alps Alpine</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Documenté</t>
+          <t>Vu</t>
         </is>
       </c>
       <c r="E23" s="7" t="n"/>
       <c r="F23" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/ProductDetail/TE-Connectivity-Linx-Technologies/ANT-868-JJB-ST?qs=K5ta8V%2BWhtbjRn899xwLFw%3D%3D</t>
+          <t>https://www.mouser.com/ProductDetail/Alps-Alpine/SKRPACE010?qs=dHDuPHwQO79W8iY66hDbLQ%3D%3D</t>
         </is>
       </c>
       <c r="G23" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=ANT-868-JJB-ST</t>
+          <t>https://www.mouser.fr/c/?q=SKRPACE010</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>Antenne UHF planaire CMS</t>
+          <t>Bouton poussoir traversant 6 × 6 mm</t>
         </is>
       </c>
       <c r="B24" s="10" t="inlineStr">
         <is>
-          <t>ANT-868-SP</t>
+          <t>B3F-1000</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>TE / Linx</t>
+          <t>Omron</t>
         </is>
       </c>
       <c r="D24" s="11" t="inlineStr">
         <is>
-          <t>Documenté</t>
+          <t>À confirmer</t>
         </is>
       </c>
       <c r="E24" s="7" t="n"/>
       <c r="F24" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/ProductDetail/Linx-Technologies/ANT-868-SP?qs=K5ta8V%2BWhtYLcp%2FwdgtLaA%3D%3D</t>
+          <t>https://www.mouser.com/ProductDetail/Omron-Electronics/B3F-1000?qs=lK7M36XCk6JQHckSc1xIsg%3D%3D</t>
         </is>
       </c>
       <c r="G24" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=ANT-868-SP</t>
+          <t>https://www.mouser.fr/c/?q=B3F-1000</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>Antennes 868 MHz — catalogue</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>Antenne UHF hélicoïdale CMS</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>ANT-868-VHETH</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>TE / Linx</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Catalogue</t>
+          <t>Documenté</t>
         </is>
       </c>
       <c r="E25" s="7" t="n"/>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/c/passive-components/antennas/?center+frequency=868+MHz</t>
+          <t>https://www.mouser.com/ProductDetail/TE-Connectivity-Linx-Technologies/ANT-868-VHETH?qs=pUKx8fyJudBCulCrBA9DxA%3D%3D</t>
         </is>
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=antenne+868+MHz</t>
+          <t>https://www.mouser.fr/c/?q=ANT-868-VHETH</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>Inductance blindée 4,7 µH, 4×4 mm (étage boost)</t>
+          <t>Antenne UHF monopole embarqué Ø7 mm</t>
         </is>
       </c>
       <c r="B26" s="10" t="inlineStr">
         <is>
-          <t>SRN4018-4R7M</t>
+          <t>ANT-868-JJB-ST</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Bourns</t>
+          <t>TE / Linx</t>
         </is>
       </c>
       <c r="D26" s="11" t="inlineStr">
         <is>
-          <t>Vu</t>
+          <t>Documenté</t>
         </is>
       </c>
       <c r="E26" s="7" t="n"/>
       <c r="F26" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/en/ProductDetail/Bourns/SRN4018-4R7M?qs=UvjENeDOEed%2FCjy5nMh3Xg%3D%3D</t>
+          <t>https://www.mouser.com/ProductDetail/TE-Connectivity-Linx-Technologies/ANT-868-JJB-ST?qs=K5ta8V%2BWhtbjRn899xwLFw%3D%3D</t>
         </is>
       </c>
       <c r="G26" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=SRN4018-4R7M</t>
+          <t>https://www.mouser.fr/c/?q=ANT-868-JJB-ST</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Condensateurs MLCC CMS — catalogue</t>
+          <t>Antenne UHF planaire CMS</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>0603 / 0805 / 1206</t>
+          <t>ANT-868-SP</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Murata, Yageo, KEMET</t>
+          <t>TE / Linx</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>Vu</t>
+          <t>Documenté</t>
         </is>
       </c>
       <c r="E27" s="7" t="n"/>
       <c r="F27" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/c/passive-components/capacitors/ceramic-capacitors/mlccs-smd-smt/</t>
+          <t>https://www.mouser.com/ProductDetail/Linx-Technologies/ANT-868-SP?qs=K5ta8V%2BWhtYLcp%2FwdgtLaA%3D%3D</t>
         </is>
       </c>
       <c r="G27" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=MLCC+0805</t>
+          <t>https://www.mouser.fr/c/?q=ANT-868-SP</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
         <is>
-          <t>Kits de condensateurs</t>
+          <t>Antennes 868 MHz — catalogue</t>
         </is>
       </c>
       <c r="B28" s="11" t="inlineStr">
@@ -1370,29 +1370,29 @@
       <c r="E28" s="7" t="n"/>
       <c r="F28" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/Passive-Components/Capacitors/Capacitor-Kits/_/N-2iq32</t>
+          <t>https://www.mouser.com/c/passive-components/antennas/?center+frequency=868+MHz</t>
         </is>
       </c>
       <c r="G28" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=capacitor+kit</t>
+          <t>https://www.mouser.fr/c/?q=antenne+868+MHz</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>Résistances CMS — catalogue</t>
+          <t>Inductance blindée 4,7 µH, 4×4 mm (étage boost)</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>RC0805 / CRCW0805</t>
+          <t>SRN4018-4R7M</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
         <is>
-          <t>Yageo, Vishay</t>
+          <t>Bourns</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
@@ -1403,116 +1403,215 @@
       <c r="E29" s="7" t="n"/>
       <c r="F29" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/c/passive-components/resistors/chip-smd-resistors/</t>
+          <t>https://www.mouser.com/en/ProductDetail/Bourns/SRN4018-4R7M?qs=UvjENeDOEed%2FCjy5nMh3Xg%3D%3D</t>
         </is>
       </c>
       <c r="G29" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=RC0805+resistance</t>
+          <t>https://www.mouser.fr/c/?q=SRN4018-4R7M</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>Kits de résistances CMS</t>
-        </is>
-      </c>
-      <c r="B30" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>Condensateurs MLCC CMS — catalogue</t>
+        </is>
+      </c>
+      <c r="B30" s="10" t="inlineStr">
+        <is>
+          <t>0603 / 0805 / 1206</t>
         </is>
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Murata, Yageo, KEMET</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr">
         <is>
-          <t>Catalogue</t>
+          <t>Vu</t>
         </is>
       </c>
       <c r="E30" s="7" t="n"/>
       <c r="F30" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/c/passive-components/resistors/resistor-kits/?termination+style=SMD%2FSMT</t>
+          <t>https://www.mouser.com/c/passive-components/capacitors/ceramic-capacitors/mlccs-smd-smt/</t>
         </is>
       </c>
       <c r="G30" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=resistor+kit+0805</t>
+          <t>https://www.mouser.fr/c/?q=MLCC+0805</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>Accus AA Ni-MH — la réparation la plus probable</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>gamme Ni-MH</t>
+          <t>Kits de condensateurs</t>
+        </is>
+      </c>
+      <c r="B31" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
         <is>
-          <t>Panasonic</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D31" s="6" t="inlineStr">
         <is>
-          <t>Prioritaire</t>
+          <t>Catalogue</t>
         </is>
       </c>
       <c r="E31" s="7" t="n"/>
       <c r="F31" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.com/en/c/power/batteries/nimh-nickel-metal-hydride-battery/?m=Panasonic</t>
+          <t>https://www.mouser.com/Passive-Components/Capacitors/Capacitor-Kits/_/N-2iq32</t>
         </is>
       </c>
       <c r="G31" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=Panasonic+NiMH+AA</t>
+          <t>https://www.mouser.fr/c/?q=capacitor+kit</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>MCU TI MSP430FR2xxx — famille</t>
+          <t>Résistances CMS — catalogue</t>
         </is>
       </c>
       <c r="B32" s="10" t="inlineStr">
         <is>
-          <t>réf. exacte à relire sur la puce</t>
+          <t>RC0805 / CRCW0805</t>
         </is>
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Texas Instruments</t>
+          <t>Yageo, Vishay</t>
         </is>
       </c>
       <c r="D32" s="11" t="inlineStr">
         <is>
-          <t>À confirmer</t>
+          <t>Vu</t>
         </is>
       </c>
       <c r="E32" s="7" t="n"/>
       <c r="F32" s="12" t="inlineStr">
         <is>
+          <t>https://www.mouser.com/c/passive-components/resistors/chip-smd-resistors/</t>
+        </is>
+      </c>
+      <c r="G32" s="12" t="inlineStr">
+        <is>
+          <t>https://www.mouser.fr/c/?q=RC0805+resistance</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>Kits de résistances CMS</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>Catalogue</t>
+        </is>
+      </c>
+      <c r="E33" s="7" t="n"/>
+      <c r="F33" s="8" t="inlineStr">
+        <is>
+          <t>https://www.mouser.com/c/passive-components/resistors/resistor-kits/?termination+style=SMD%2FSMT</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
+          <t>https://www.mouser.fr/c/?q=resistor+kit+0805</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>Accus AA Ni-MH — la réparation la plus probable</t>
+        </is>
+      </c>
+      <c r="B34" s="10" t="inlineStr">
+        <is>
+          <t>gamme Ni-MH</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>Panasonic</t>
+        </is>
+      </c>
+      <c r="D34" s="11" t="inlineStr">
+        <is>
+          <t>Prioritaire</t>
+        </is>
+      </c>
+      <c r="E34" s="7" t="n"/>
+      <c r="F34" s="12" t="inlineStr">
+        <is>
+          <t>https://www.mouser.com/en/c/power/batteries/nimh-nickel-metal-hydride-battery/?m=Panasonic</t>
+        </is>
+      </c>
+      <c r="G34" s="12" t="inlineStr">
+        <is>
+          <t>https://www.mouser.fr/c/?q=Panasonic+NiMH+AA</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>MCU TI MSP430FR2xxx — famille</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>réf. exacte à relire sur la puce</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>Texas Instruments</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>À confirmer</t>
+        </is>
+      </c>
+      <c r="E35" s="7" t="n"/>
+      <c r="F35" s="8" t="inlineStr">
+        <is>
           <t>https://www.mouser.com/c/semiconductors/embedded-processors-controllers/microcontrollers-mcu/?q=MSP430FR2</t>
         </is>
       </c>
-      <c r="G32" s="12" t="inlineStr">
+      <c r="G35" s="8" t="inlineStr">
         <is>
           <t>https://www.mouser.fr/c/?q=MSP430FR2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G32"/>
+  <autoFilter ref="A4:G35"/>
   <mergeCells count="2">
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A1:G1"/>
@@ -1574,6 +1673,12 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId54"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId55"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId62"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1807,7 +1912,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Diamètre extérieur de la bague en façade : ~12,9 mm avec corps ~15 × 17 mm → série KPJX ; ~9,5 mm → mini-DIN, autre famille limitée à ~1 A. Puis compter les trous côté cuivre : 4 contacts + 2 ergots + languette de masse → version blindée.</t>
+          <t>Plan de perçage constructeur à comparer trou par trou : https://www.mouser.com/datasheet/3/166/1/KPJX.pdf  —  Diamètre extérieur de la bague en façade : ~12,9 mm avec corps ~15 × 17 mm → série KPJX ; ~9,5 mm → mini-DIN, autre famille limitée à ~1 A. Puis compter les trous côté cuivre : 4 contacts + 2 ergots + languette de masse → version blindée.</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Lead with the token-free search link, and record why
Testing the URLs with curl returns 403 on the CONNECT tunnel for both
www.mouser.fr and www.mouser.com: an organisation egress policy denial,
so no Mouser link can be verified from this session at all — worth
stating rather than working around.

The user's own screenshot shows the likely breakage: a mouser.com
product URL lands on mouser.fr/fr/ProductDetail/... with the ?qs= token
stripped, which is a 404. The search-by-reference URL depends on no
token, so it now leads as the primary link column and the direct product
page moves to second.

CLAUDE.md records the redirect behaviour, the verified egress denial, and
the rule that the manufacturer reference — not the URL — is the durable
identifier a parts list must carry.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ge7EoEedmTKdVGHi238WWF
</commit_message>
<xml_diff>
--- a/exports/Liste-Mouser-Tonwelt-TG288.xlsx
+++ b/exports/Liste-Mouser-Tonwelt-TG288.xlsx
@@ -528,12 +528,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
-    <col width="62" customWidth="1" min="6" max="6"/>
-    <col width="44" customWidth="1" min="7" max="7"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="62" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -578,12 +578,12 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Lien produit Mouser</t>
+          <t>Recherche Mouser (lien fiable)</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Recherche par référence</t>
+          <t>Fiche produit (si elle répond)</t>
         </is>
       </c>
     </row>
@@ -611,12 +611,12 @@
       <c r="E5" s="7" t="n"/>
       <c r="F5" s="8" t="inlineStr">
         <is>
+          <t>https://www.mouser.fr/c/?q=KPJX-4S-S</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
           <t>https://www.mouser.com/en/ProductDetail/Kycon/KPJX-4S-S?qs=0QDpPFt3C4bj8uE5yBzCJQ%3D%3D</t>
-        </is>
-      </c>
-      <c r="G5" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=KPJX-4S-S</t>
         </is>
       </c>
     </row>
@@ -644,12 +644,12 @@
       <c r="E6" s="7" t="n"/>
       <c r="F6" s="12" t="inlineStr">
         <is>
+          <t>https://www.mouser.fr/c/?q=KPJX-4S</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="inlineStr">
+        <is>
           <t>https://www.mouser.fr/ProductDetail/Kycon/KPJX-4S?qs=PGF6ObTbUZ1PHc9As62%2FZQ%3D%3D</t>
-        </is>
-      </c>
-      <c r="G6" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=KPJX-4S</t>
         </is>
       </c>
     </row>
@@ -677,12 +677,12 @@
       <c r="E7" s="7" t="n"/>
       <c r="F7" s="8" t="inlineStr">
         <is>
+          <t>https://www.mouser.fr/c/?q=KPJX-PM-4S-S</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
           <t>https://www.mouser.com/ProductDetail/Kycon/KPJX-PM-4S-S?qs=zorda86t5M9ArIfKgei5Pg%3D%3D</t>
-        </is>
-      </c>
-      <c r="G7" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=KPJX-PM-4S-S</t>
         </is>
       </c>
     </row>
@@ -710,12 +710,12 @@
       <c r="E8" s="7" t="n"/>
       <c r="F8" s="12" t="inlineStr">
         <is>
+          <t>https://www.mouser.fr/c/?q=KPJ-4S</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
           <t>https://www.mouser.com/ProductDetail/Kycon/KPJ-4S?qs=/XicOQBKAMa%252BcJ0hGGZaig%3D%3D</t>
-        </is>
-      </c>
-      <c r="G8" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=KPJ-4S</t>
         </is>
       </c>
     </row>
@@ -743,12 +743,12 @@
       <c r="E9" s="7" t="n"/>
       <c r="F9" s="8" t="inlineStr">
         <is>
+          <t>https://www.mouser.fr/c/?q=KPJ-4S-S</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
           <t>https://www.mouser.com/ProductDetail/Kycon/KPJ-4S-S?qs=SrUfdAPSdgAPLkBk%2BStEGA%3D%3D</t>
-        </is>
-      </c>
-      <c r="G9" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=KPJ-4S-S</t>
         </is>
       </c>
     </row>
@@ -776,12 +776,12 @@
       <c r="E10" s="7" t="n"/>
       <c r="F10" s="12" t="inlineStr">
         <is>
+          <t>https://www.mouser.fr/c/?q=KPJXHT-4S-S</t>
+        </is>
+      </c>
+      <c r="G10" s="12" t="inlineStr">
+        <is>
           <t>https://www.mouser.com/ProductDetail/Kycon/KPJXHT-4S-S?qs=6olcXJbp99TwdwXWG%2BzyAQ%3D%3D</t>
-        </is>
-      </c>
-      <c r="G10" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=KPJXHT-4S-S</t>
         </is>
       </c>
     </row>
@@ -809,12 +809,12 @@
       <c r="E11" s="7" t="n"/>
       <c r="F11" s="8" t="inlineStr">
         <is>
+          <t>https://www.mouser.fr/c/?q=KPPX-4P</t>
+        </is>
+      </c>
+      <c r="G11" s="8" t="inlineStr">
+        <is>
           <t>https://www.mouser.com/ProductDetail/Kycon/KPPX-4P?qs=Y0vc5luVLxJNKFay3ZyJLw%3D%3D</t>
-        </is>
-      </c>
-      <c r="G11" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=KPPX-4P</t>
         </is>
       </c>
     </row>
@@ -842,12 +842,12 @@
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="12" t="inlineStr">
         <is>
+          <t>https://www.mouser.fr/c/?q=SJ-43514</t>
+        </is>
+      </c>
+      <c r="G12" s="12" t="inlineStr">
+        <is>
           <t>https://www.mouser.com/ProductDetail/Same-Sky/SJ-43514?qs=WyjlAZoYn51bsBOfuwwiuw%3D%3D</t>
-        </is>
-      </c>
-      <c r="G12" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=SJ-43514</t>
         </is>
       </c>
     </row>
@@ -875,12 +875,12 @@
       <c r="E13" s="7" t="n"/>
       <c r="F13" s="8" t="inlineStr">
         <is>
+          <t>https://www.mouser.fr/c/?q=SJ-43514-SMT-TR</t>
+        </is>
+      </c>
+      <c r="G13" s="8" t="inlineStr">
+        <is>
           <t>https://www.mouser.com/ProductDetail/CUI-Devices/SJ-43514-SMT-TR/?qs=WyjlAZoYn528%252BiAb5RzVtg%3D%3D</t>
-        </is>
-      </c>
-      <c r="G13" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=SJ-43514-SMT-TR</t>
         </is>
       </c>
     </row>
@@ -908,12 +908,12 @@
       <c r="E14" s="7" t="n"/>
       <c r="F14" s="12" t="inlineStr">
         <is>
+          <t>https://www.mouser.fr/c/?q=10118193-0001LF</t>
+        </is>
+      </c>
+      <c r="G14" s="12" t="inlineStr">
+        <is>
           <t>https://www.mouser.com/ProductDetail/Amphenol-FCI/10118193-0001LF?qs=Ywefl8B65e63Nsqd%2B8HZaQ%3D%3D</t>
-        </is>
-      </c>
-      <c r="G14" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=10118193-0001LF</t>
         </is>
       </c>
     </row>
@@ -941,12 +941,12 @@
       <c r="E15" s="7" t="n"/>
       <c r="F15" s="8" t="inlineStr">
         <is>
+          <t>https://www.mouser.fr/c/?q=10118192-0001LF</t>
+        </is>
+      </c>
+      <c r="G15" s="8" t="inlineStr">
+        <is>
           <t>https://www.mouser.com/ProductDetail/Amphenol-FCI/10118192-0001LF?qs=Ywefl8B65e5bHFoQtIudZg%3D%3D</t>
-        </is>
-      </c>
-      <c r="G15" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=10118192-0001LF</t>
         </is>
       </c>
     </row>
@@ -974,12 +974,12 @@
       <c r="E16" s="7" t="n"/>
       <c r="F16" s="12" t="inlineStr">
         <is>
+          <t>https://www.mouser.fr/c/?q=10118194-0001LF</t>
+        </is>
+      </c>
+      <c r="G16" s="12" t="inlineStr">
+        <is>
           <t>https://www.mouser.com/en/ProductDetail/Amphenol-FCI/10118194-0001LF?qs=Ywefl8B65e4FIdY8OWfRQA%3D%3D</t>
-        </is>
-      </c>
-      <c r="G16" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=10118194-0001LF</t>
         </is>
       </c>
     </row>
@@ -1007,12 +1007,12 @@
       <c r="E17" s="7" t="n"/>
       <c r="F17" s="8" t="inlineStr">
         <is>
+          <t>https://www.mouser.fr/c/?q=54819-0519</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
           <t>https://www.mouser.com/ProductDetail/Molex/54819-0519?qs=x6EjVpvqMVObi%2BAAyuuEww%3D%3D</t>
-        </is>
-      </c>
-      <c r="G17" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=54819-0519</t>
         </is>
       </c>
     </row>
@@ -1040,12 +1040,12 @@
       <c r="E18" s="7" t="n"/>
       <c r="F18" s="12" t="inlineStr">
         <is>
+          <t>https://www.mouser.fr/c/?q=USB4085-GF-A</t>
+        </is>
+      </c>
+      <c r="G18" s="12" t="inlineStr">
+        <is>
           <t>https://www.mouser.com/ProductDetail/GCT/USB4085-GF-A?qs=KUoIvG%2F9Ilba1bQOahfWjw%3D%3D</t>
-        </is>
-      </c>
-      <c r="G18" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=USB4085-GF-A</t>
         </is>
       </c>
     </row>
@@ -1073,12 +1073,12 @@
       <c r="E19" s="7" t="n"/>
       <c r="F19" s="8" t="inlineStr">
         <is>
+          <t>https://www.mouser.fr/c/?q=MF-MSMF</t>
+        </is>
+      </c>
+      <c r="G19" s="8" t="inlineStr">
+        <is>
           <t>https://www.mouser.com/new/bourns/bourns-mf-msmf-series-fuses/</t>
-        </is>
-      </c>
-      <c r="G19" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=MF-MSMF</t>
         </is>
       </c>
     </row>
@@ -1106,12 +1106,12 @@
       <c r="E20" s="7" t="n"/>
       <c r="F20" s="12" t="inlineStr">
         <is>
+          <t>https://www.mouser.fr/c/?q=fusible+PPTC+1812</t>
+        </is>
+      </c>
+      <c r="G20" s="12" t="inlineStr">
+        <is>
           <t>https://www.mouser.com/c/circuit-protection/thermistors/resettable-fuses-pptc/</t>
-        </is>
-      </c>
-      <c r="G20" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=fusible+PPTC+1812</t>
         </is>
       </c>
     </row>
@@ -1139,12 +1139,12 @@
       <c r="E21" s="7" t="n"/>
       <c r="F21" s="8" t="inlineStr">
         <is>
+          <t>https://www.mouser.fr/c/?q=AS01508MR-6-R</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
+        <is>
           <t>https://www.mouser.com/ProductDetail/PUI-Audio/AS01508MR-6-R?qs=vgjKjNJexThgIp5KgUGpgA%3D%3D</t>
-        </is>
-      </c>
-      <c r="G21" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=AS01508MR-6-R</t>
         </is>
       </c>
     </row>
@@ -1172,12 +1172,12 @@
       <c r="E22" s="7" t="n"/>
       <c r="F22" s="12" t="inlineStr">
         <is>
+          <t>https://www.mouser.fr/c/?q=haut-parleur+15mm+8+ohm</t>
+        </is>
+      </c>
+      <c r="G22" s="12" t="inlineStr">
+        <is>
           <t>https://www.mouser.com/en/c/electromechanical/audio-devices/speakers-transducers/</t>
-        </is>
-      </c>
-      <c r="G22" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=haut-parleur+15mm+8+ohm</t>
         </is>
       </c>
     </row>
@@ -1205,12 +1205,12 @@
       <c r="E23" s="7" t="n"/>
       <c r="F23" s="8" t="inlineStr">
         <is>
+          <t>https://www.mouser.fr/c/?q=SKRPACE010</t>
+        </is>
+      </c>
+      <c r="G23" s="8" t="inlineStr">
+        <is>
           <t>https://www.mouser.com/ProductDetail/Alps-Alpine/SKRPACE010?qs=dHDuPHwQO79W8iY66hDbLQ%3D%3D</t>
-        </is>
-      </c>
-      <c r="G23" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=SKRPACE010</t>
         </is>
       </c>
     </row>
@@ -1238,12 +1238,12 @@
       <c r="E24" s="7" t="n"/>
       <c r="F24" s="12" t="inlineStr">
         <is>
+          <t>https://www.mouser.fr/c/?q=B3F-1000</t>
+        </is>
+      </c>
+      <c r="G24" s="12" t="inlineStr">
+        <is>
           <t>https://www.mouser.com/ProductDetail/Omron-Electronics/B3F-1000?qs=lK7M36XCk6JQHckSc1xIsg%3D%3D</t>
-        </is>
-      </c>
-      <c r="G24" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=B3F-1000</t>
         </is>
       </c>
     </row>
@@ -1271,12 +1271,12 @@
       <c r="E25" s="7" t="n"/>
       <c r="F25" s="8" t="inlineStr">
         <is>
+          <t>https://www.mouser.fr/c/?q=ANT-868-VHETH</t>
+        </is>
+      </c>
+      <c r="G25" s="8" t="inlineStr">
+        <is>
           <t>https://www.mouser.com/ProductDetail/TE-Connectivity-Linx-Technologies/ANT-868-VHETH?qs=pUKx8fyJudBCulCrBA9DxA%3D%3D</t>
-        </is>
-      </c>
-      <c r="G25" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=ANT-868-VHETH</t>
         </is>
       </c>
     </row>
@@ -1304,12 +1304,12 @@
       <c r="E26" s="7" t="n"/>
       <c r="F26" s="12" t="inlineStr">
         <is>
+          <t>https://www.mouser.fr/c/?q=ANT-868-JJB-ST</t>
+        </is>
+      </c>
+      <c r="G26" s="12" t="inlineStr">
+        <is>
           <t>https://www.mouser.com/ProductDetail/TE-Connectivity-Linx-Technologies/ANT-868-JJB-ST?qs=K5ta8V%2BWhtbjRn899xwLFw%3D%3D</t>
-        </is>
-      </c>
-      <c r="G26" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=ANT-868-JJB-ST</t>
         </is>
       </c>
     </row>
@@ -1337,12 +1337,12 @@
       <c r="E27" s="7" t="n"/>
       <c r="F27" s="8" t="inlineStr">
         <is>
+          <t>https://www.mouser.fr/c/?q=ANT-868-SP</t>
+        </is>
+      </c>
+      <c r="G27" s="8" t="inlineStr">
+        <is>
           <t>https://www.mouser.com/ProductDetail/Linx-Technologies/ANT-868-SP?qs=K5ta8V%2BWhtYLcp%2FwdgtLaA%3D%3D</t>
-        </is>
-      </c>
-      <c r="G27" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=ANT-868-SP</t>
         </is>
       </c>
     </row>
@@ -1370,12 +1370,12 @@
       <c r="E28" s="7" t="n"/>
       <c r="F28" s="12" t="inlineStr">
         <is>
+          <t>https://www.mouser.fr/c/?q=antenne+868+MHz</t>
+        </is>
+      </c>
+      <c r="G28" s="12" t="inlineStr">
+        <is>
           <t>https://www.mouser.com/c/passive-components/antennas/?center+frequency=868+MHz</t>
-        </is>
-      </c>
-      <c r="G28" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=antenne+868+MHz</t>
         </is>
       </c>
     </row>
@@ -1403,12 +1403,12 @@
       <c r="E29" s="7" t="n"/>
       <c r="F29" s="8" t="inlineStr">
         <is>
+          <t>https://www.mouser.fr/c/?q=SRN4018-4R7M</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
           <t>https://www.mouser.com/en/ProductDetail/Bourns/SRN4018-4R7M?qs=UvjENeDOEed%2FCjy5nMh3Xg%3D%3D</t>
-        </is>
-      </c>
-      <c r="G29" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=SRN4018-4R7M</t>
         </is>
       </c>
     </row>
@@ -1436,12 +1436,12 @@
       <c r="E30" s="7" t="n"/>
       <c r="F30" s="12" t="inlineStr">
         <is>
+          <t>https://www.mouser.fr/c/?q=MLCC+0805</t>
+        </is>
+      </c>
+      <c r="G30" s="12" t="inlineStr">
+        <is>
           <t>https://www.mouser.com/c/passive-components/capacitors/ceramic-capacitors/mlccs-smd-smt/</t>
-        </is>
-      </c>
-      <c r="G30" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=MLCC+0805</t>
         </is>
       </c>
     </row>
@@ -1469,12 +1469,12 @@
       <c r="E31" s="7" t="n"/>
       <c r="F31" s="8" t="inlineStr">
         <is>
+          <t>https://www.mouser.fr/c/?q=capacitor+kit</t>
+        </is>
+      </c>
+      <c r="G31" s="8" t="inlineStr">
+        <is>
           <t>https://www.mouser.com/Passive-Components/Capacitors/Capacitor-Kits/_/N-2iq32</t>
-        </is>
-      </c>
-      <c r="G31" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=capacitor+kit</t>
         </is>
       </c>
     </row>
@@ -1502,12 +1502,12 @@
       <c r="E32" s="7" t="n"/>
       <c r="F32" s="12" t="inlineStr">
         <is>
+          <t>https://www.mouser.fr/c/?q=RC0805+resistance</t>
+        </is>
+      </c>
+      <c r="G32" s="12" t="inlineStr">
+        <is>
           <t>https://www.mouser.com/c/passive-components/resistors/chip-smd-resistors/</t>
-        </is>
-      </c>
-      <c r="G32" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=RC0805+resistance</t>
         </is>
       </c>
     </row>
@@ -1535,12 +1535,12 @@
       <c r="E33" s="7" t="n"/>
       <c r="F33" s="8" t="inlineStr">
         <is>
+          <t>https://www.mouser.fr/c/?q=resistor+kit+0805</t>
+        </is>
+      </c>
+      <c r="G33" s="8" t="inlineStr">
+        <is>
           <t>https://www.mouser.com/c/passive-components/resistors/resistor-kits/?termination+style=SMD%2FSMT</t>
-        </is>
-      </c>
-      <c r="G33" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=resistor+kit+0805</t>
         </is>
       </c>
     </row>
@@ -1568,12 +1568,12 @@
       <c r="E34" s="7" t="n"/>
       <c r="F34" s="12" t="inlineStr">
         <is>
+          <t>https://www.mouser.fr/c/?q=Panasonic+NiMH+AA</t>
+        </is>
+      </c>
+      <c r="G34" s="12" t="inlineStr">
+        <is>
           <t>https://www.mouser.com/en/c/power/batteries/nimh-nickel-metal-hydride-battery/?m=Panasonic</t>
-        </is>
-      </c>
-      <c r="G34" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=Panasonic+NiMH+AA</t>
         </is>
       </c>
     </row>
@@ -1601,12 +1601,12 @@
       <c r="E35" s="7" t="n"/>
       <c r="F35" s="8" t="inlineStr">
         <is>
+          <t>https://www.mouser.fr/c/?q=MSP430FR2</t>
+        </is>
+      </c>
+      <c r="G35" s="8" t="inlineStr">
+        <is>
           <t>https://www.mouser.com/c/semiconductors/embedded-processors-controllers/microcontrollers-mcu/?q=MSP430FR2</t>
-        </is>
-      </c>
-      <c r="G35" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=MSP430FR2</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Standardise every Mouser link on the search form that works
The user confirmed https://www.mouser.fr/c/?q=<REF> resolves, so that is
now the only link form anywhere: 31 rows in the workbook, one link column
instead of two, and 66 dead ProductDetail URLs rewritten across the three
sourcing notes.

Converting the docs needed a second pass — the first rule stripped a
leading digit group meant for Mouser's own part numbers (490-SJ-43514)
and mangled two manufacturer references into 0001LF and 0519. It now
takes the last path segment when a manufacturer directory is present and
only strips a three-digit Mouser prefix otherwise; all 30 rewritten
references were checked one by one.

CLAUDE.md drops the "search first, product page second" wording for a
plain ban on shipping ProductDetail URLs at all.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ge7EoEedmTKdVGHi238WWF
</commit_message>
<xml_diff>
--- a/exports/Liste-Mouser-Tonwelt-TG288.xlsx
+++ b/exports/Liste-Mouser-Tonwelt-TG288.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Sources &amp; statuts" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Liste Mouser'!$A$4:$G$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Liste Mouser'!$A$4:$F$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -524,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -532,8 +532,7 @@
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
-    <col width="44" customWidth="1" min="6" max="6"/>
-    <col width="62" customWidth="1" min="7" max="7"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -578,12 +577,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Recherche Mouser (lien fiable)</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Fiche produit (si elle répond)</t>
+          <t>Lien Mouser (recherche par référence)</t>
         </is>
       </c>
     </row>
@@ -614,11 +608,6 @@
           <t>https://www.mouser.fr/c/?q=KPJX-4S-S</t>
         </is>
       </c>
-      <c r="G5" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/en/ProductDetail/Kycon/KPJX-4S-S?qs=0QDpPFt3C4bj8uE5yBzCJQ%3D%3D</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
@@ -647,11 +636,6 @@
           <t>https://www.mouser.fr/c/?q=KPJX-4S</t>
         </is>
       </c>
-      <c r="G6" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/ProductDetail/Kycon/KPJX-4S?qs=PGF6ObTbUZ1PHc9As62%2FZQ%3D%3D</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -680,11 +664,6 @@
           <t>https://www.mouser.fr/c/?q=KPJX-PM-4S-S</t>
         </is>
       </c>
-      <c r="G7" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/ProductDetail/Kycon/KPJX-PM-4S-S?qs=zorda86t5M9ArIfKgei5Pg%3D%3D</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -713,11 +692,6 @@
           <t>https://www.mouser.fr/c/?q=KPJ-4S</t>
         </is>
       </c>
-      <c r="G8" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/ProductDetail/Kycon/KPJ-4S?qs=/XicOQBKAMa%252BcJ0hGGZaig%3D%3D</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -746,11 +720,6 @@
           <t>https://www.mouser.fr/c/?q=KPJ-4S-S</t>
         </is>
       </c>
-      <c r="G9" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/ProductDetail/Kycon/KPJ-4S-S?qs=SrUfdAPSdgAPLkBk%2BStEGA%3D%3D</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -779,11 +748,6 @@
           <t>https://www.mouser.fr/c/?q=KPJXHT-4S-S</t>
         </is>
       </c>
-      <c r="G10" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/ProductDetail/Kycon/KPJXHT-4S-S?qs=6olcXJbp99TwdwXWG%2BzyAQ%3D%3D</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -812,11 +776,6 @@
           <t>https://www.mouser.fr/c/?q=KPPX-4P</t>
         </is>
       </c>
-      <c r="G11" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/ProductDetail/Kycon/KPPX-4P?qs=Y0vc5luVLxJNKFay3ZyJLw%3D%3D</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -845,11 +804,6 @@
           <t>https://www.mouser.fr/c/?q=SJ-43514</t>
         </is>
       </c>
-      <c r="G12" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/ProductDetail/Same-Sky/SJ-43514?qs=WyjlAZoYn51bsBOfuwwiuw%3D%3D</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -878,11 +832,6 @@
           <t>https://www.mouser.fr/c/?q=SJ-43514-SMT-TR</t>
         </is>
       </c>
-      <c r="G13" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/ProductDetail/CUI-Devices/SJ-43514-SMT-TR/?qs=WyjlAZoYn528%252BiAb5RzVtg%3D%3D</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
@@ -911,11 +860,6 @@
           <t>https://www.mouser.fr/c/?q=10118193-0001LF</t>
         </is>
       </c>
-      <c r="G14" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/ProductDetail/Amphenol-FCI/10118193-0001LF?qs=Ywefl8B65e63Nsqd%2B8HZaQ%3D%3D</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -944,11 +888,6 @@
           <t>https://www.mouser.fr/c/?q=10118192-0001LF</t>
         </is>
       </c>
-      <c r="G15" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/ProductDetail/Amphenol-FCI/10118192-0001LF?qs=Ywefl8B65e5bHFoQtIudZg%3D%3D</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
@@ -977,11 +916,6 @@
           <t>https://www.mouser.fr/c/?q=10118194-0001LF</t>
         </is>
       </c>
-      <c r="G16" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/en/ProductDetail/Amphenol-FCI/10118194-0001LF?qs=Ywefl8B65e4FIdY8OWfRQA%3D%3D</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -1010,11 +944,6 @@
           <t>https://www.mouser.fr/c/?q=54819-0519</t>
         </is>
       </c>
-      <c r="G17" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/ProductDetail/Molex/54819-0519?qs=x6EjVpvqMVObi%2BAAyuuEww%3D%3D</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
@@ -1043,11 +972,6 @@
           <t>https://www.mouser.fr/c/?q=USB4085-GF-A</t>
         </is>
       </c>
-      <c r="G18" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/ProductDetail/GCT/USB4085-GF-A?qs=KUoIvG%2F9Ilba1bQOahfWjw%3D%3D</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -1076,11 +1000,6 @@
           <t>https://www.mouser.fr/c/?q=MF-MSMF</t>
         </is>
       </c>
-      <c r="G19" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/new/bourns/bourns-mf-msmf-series-fuses/</t>
-        </is>
-      </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
@@ -1109,11 +1028,6 @@
           <t>https://www.mouser.fr/c/?q=fusible+PPTC+1812</t>
         </is>
       </c>
-      <c r="G20" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/c/circuit-protection/thermistors/resettable-fuses-pptc/</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
@@ -1142,11 +1056,6 @@
           <t>https://www.mouser.fr/c/?q=AS01508MR-6-R</t>
         </is>
       </c>
-      <c r="G21" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/ProductDetail/PUI-Audio/AS01508MR-6-R?qs=vgjKjNJexThgIp5KgUGpgA%3D%3D</t>
-        </is>
-      </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
@@ -1175,11 +1084,6 @@
           <t>https://www.mouser.fr/c/?q=haut-parleur+15mm+8+ohm</t>
         </is>
       </c>
-      <c r="G22" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/en/c/electromechanical/audio-devices/speakers-transducers/</t>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1208,11 +1112,6 @@
           <t>https://www.mouser.fr/c/?q=SKRPACE010</t>
         </is>
       </c>
-      <c r="G23" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/ProductDetail/Alps-Alpine/SKRPACE010?qs=dHDuPHwQO79W8iY66hDbLQ%3D%3D</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
@@ -1241,11 +1140,6 @@
           <t>https://www.mouser.fr/c/?q=B3F-1000</t>
         </is>
       </c>
-      <c r="G24" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/ProductDetail/Omron-Electronics/B3F-1000?qs=lK7M36XCk6JQHckSc1xIsg%3D%3D</t>
-        </is>
-      </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
@@ -1274,11 +1168,6 @@
           <t>https://www.mouser.fr/c/?q=ANT-868-VHETH</t>
         </is>
       </c>
-      <c r="G25" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/ProductDetail/TE-Connectivity-Linx-Technologies/ANT-868-VHETH?qs=pUKx8fyJudBCulCrBA9DxA%3D%3D</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" s="9" t="inlineStr">
@@ -1307,11 +1196,6 @@
           <t>https://www.mouser.fr/c/?q=ANT-868-JJB-ST</t>
         </is>
       </c>
-      <c r="G26" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/ProductDetail/TE-Connectivity-Linx-Technologies/ANT-868-JJB-ST?qs=K5ta8V%2BWhtbjRn899xwLFw%3D%3D</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
@@ -1340,11 +1224,6 @@
           <t>https://www.mouser.fr/c/?q=ANT-868-SP</t>
         </is>
       </c>
-      <c r="G27" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/ProductDetail/Linx-Technologies/ANT-868-SP?qs=K5ta8V%2BWhtYLcp%2FwdgtLaA%3D%3D</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
@@ -1373,11 +1252,6 @@
           <t>https://www.mouser.fr/c/?q=antenne+868+MHz</t>
         </is>
       </c>
-      <c r="G28" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/c/passive-components/antennas/?center+frequency=868+MHz</t>
-        </is>
-      </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -1406,11 +1280,6 @@
           <t>https://www.mouser.fr/c/?q=SRN4018-4R7M</t>
         </is>
       </c>
-      <c r="G29" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/en/ProductDetail/Bourns/SRN4018-4R7M?qs=UvjENeDOEed%2FCjy5nMh3Xg%3D%3D</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
@@ -1439,11 +1308,6 @@
           <t>https://www.mouser.fr/c/?q=MLCC+0805</t>
         </is>
       </c>
-      <c r="G30" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/c/passive-components/capacitors/ceramic-capacitors/mlccs-smd-smt/</t>
-        </is>
-      </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -1472,11 +1336,6 @@
           <t>https://www.mouser.fr/c/?q=capacitor+kit</t>
         </is>
       </c>
-      <c r="G31" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/Passive-Components/Capacitors/Capacitor-Kits/_/N-2iq32</t>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
@@ -1505,11 +1364,6 @@
           <t>https://www.mouser.fr/c/?q=RC0805+resistance</t>
         </is>
       </c>
-      <c r="G32" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/c/passive-components/resistors/chip-smd-resistors/</t>
-        </is>
-      </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
@@ -1538,11 +1392,6 @@
           <t>https://www.mouser.fr/c/?q=resistor+kit+0805</t>
         </is>
       </c>
-      <c r="G33" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/c/passive-components/resistors/resistor-kits/?termination+style=SMD%2FSMT</t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
@@ -1571,11 +1420,6 @@
           <t>https://www.mouser.fr/c/?q=Panasonic+NiMH+AA</t>
         </is>
       </c>
-      <c r="G34" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/en/c/power/batteries/nimh-nickel-metal-hydride-battery/?m=Panasonic</t>
-        </is>
-      </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -1604,81 +1448,45 @@
           <t>https://www.mouser.fr/c/?q=MSP430FR2</t>
         </is>
       </c>
-      <c r="G35" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.com/c/semiconductors/embedded-processors-controllers/microcontrollers-mcu/?q=MSP430FR2</t>
-        </is>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:G35"/>
+  <autoFilter ref="A4:F35"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G34" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G35" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F12" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F13" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F14" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F15" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F16" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F17" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId31"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rebuild the list from the user's own selection
The user returned the workbook trimmed to the 16 lines they judged
relevant, so that selection — not mine — is now the script's row list:
the shielded Kycon inlet and its mating plug, the surface-mount jack,
three micro-USB variants, the mini-USB, the PPTC fuse, the speaker and
antenna families, the boost inductor, the MLCC and resistor-kit
catalogues, and the MSP430 family.

Added on top, as requested: the low-profile Alps SKRW tact switches with
the landing page the user supplied plus its life-rating variants, and a
flat lithium cell replacing the NiMH row.

Also drops TG-288 from the sheet title. Which model the fleet actually
uses is still unanswered, and the earlier title asserted it.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ge7EoEedmTKdVGHi238WWF
</commit_message>
<xml_diff>
--- a/exports/Liste-Mouser-Tonwelt-TG288.xlsx
+++ b/exports/Liste-Mouser-Tonwelt-TG288.xlsx
@@ -13,7 +13,7 @@
     <sheet name="Sources &amp; statuts" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Liste Mouser'!$A$4:$F$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Liste Mouser'!$A$4:$F$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -524,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -538,14 +538,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Liste Mouser — audioguide Tonwelt / Linkx TG-288 et sa valise de charge</t>
+          <t>Liste Mouser — audioguide Tonwelt / Linkx et sa valise de charge</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Prix et stocks volontairement absents : ils changent — à lire sur la page produit au moment de commander.  Colonne E (Qté) en jaune : à compléter, nombre entier, ex. 2.  Colonne F : adresse en clair, à copier-coller.  Colonne G : cliquer sur « Ouvrir ».</t>
+          <t>Liste arrêtée par l'utilisateur (16 lignes retenues sur 31), plus les poussoirs SKRW et la batterie lithium.  Prix et stocks absents : ils changent.  Colonne E (Qté) en jaune : à compléter, nombre entier, ex. 2.  Colonne F : adresse en clair, à copier-coller.  Colonne G : cliquer sur « Ouvrir ».</t>
         </is>
       </c>
     </row>
@@ -612,12 +612,12 @@
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t>Prise alimentation DIN puissance 4 contacts, non blindée</t>
+          <t>Fiche mâle d'accouplement (réfection du cordon)</t>
         </is>
       </c>
       <c r="B6" s="10" t="inlineStr">
         <is>
-          <t>KPJX-4S</t>
+          <t>KPPX-4P</t>
         </is>
       </c>
       <c r="C6" s="11" t="inlineStr">
@@ -633,108 +633,108 @@
       <c r="E6" s="7" t="n"/>
       <c r="F6" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=KPJX-4S</t>
+          <t>https://www.mouser.fr/c/?q=KPPX-4P</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Prise alimentation, montage sur panneau</t>
+          <t>Prise jack 3,5 mm, CMS</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>KPJX-PM-4S-S</t>
+          <t>SJ-43514-SMT-TR</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Kycon</t>
+          <t>Same Sky (CUI Devices)</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Variante</t>
+          <t>Documenté</t>
         </is>
       </c>
       <c r="E7" s="7" t="n"/>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=KPJX-PM-4S-S</t>
+          <t>https://www.mouser.fr/c/?q=SJ-43514-SMT-TR</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>Prise alimentation DIN puissance 4 contacts — série voisine KPJ, non blindée</t>
+          <t>Micro-USB B, CMS coudée</t>
         </is>
       </c>
       <c r="B8" s="10" t="inlineStr">
         <is>
-          <t>KPJ-4S</t>
+          <t>10118193-0001LF</t>
         </is>
       </c>
       <c r="C8" s="11" t="inlineStr">
         <is>
-          <t>Kycon</t>
+          <t>Amphenol FCI</t>
         </is>
       </c>
       <c r="D8" s="11" t="inlineStr">
         <is>
-          <t>À départager</t>
+          <t>Documenté</t>
         </is>
       </c>
       <c r="E8" s="7" t="n"/>
       <c r="F8" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=KPJ-4S</t>
+          <t>https://www.mouser.fr/c/?q=10118193-0001LF</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Prise alimentation DIN puissance 4 contacts — série voisine KPJ, blindée</t>
+          <t>Micro-USB B, variante de montage</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>KPJ-4S-S</t>
+          <t>10118192-0001LF</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Kycon</t>
+          <t>Amphenol FCI</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>À départager</t>
+          <t>Variante</t>
         </is>
       </c>
       <c r="E9" s="7" t="n"/>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=KPJ-4S-S</t>
+          <t>https://www.mouser.fr/c/?q=10118192-0001LF</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t>Prise alimentation DIN puissance 4 contacts — version haute température</t>
+          <t>Micro-USB B, variante de montage</t>
         </is>
       </c>
       <c r="B10" s="10" t="inlineStr">
         <is>
-          <t>KPJXHT-4S-S</t>
+          <t>10118194-0001LF</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
         <is>
-          <t>Kycon</t>
+          <t>Amphenol FCI</t>
         </is>
       </c>
       <c r="D10" s="11" t="inlineStr">
@@ -745,322 +745,322 @@
       <c r="E10" s="7" t="n"/>
       <c r="F10" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=KPJXHT-4S-S</t>
+          <t>https://www.mouser.fr/c/?q=10118194-0001LF</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Fiche mâle d'accouplement (réfection du cordon)</t>
+          <t>Mini-USB B, 5 contacts</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>KPPX-4P</t>
+          <t>54819-0519</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Kycon</t>
+          <t>Molex</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Variante</t>
+          <t>À confirmer</t>
         </is>
       </c>
       <c r="E11" s="7" t="n"/>
       <c r="F11" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=KPPX-4P</t>
+          <t>https://www.mouser.fr/c/?q=54819-0519</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>Prise jack 3,5 mm, traversante</t>
+          <t>Poussoir tactile CMS bas profil — série SKRW</t>
         </is>
       </c>
       <c r="B12" s="10" t="inlineStr">
         <is>
-          <t>SJ-43514</t>
+          <t>série SKRW</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Same Sky (CUI Devices)</t>
+          <t>Alps Alpine</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>Documenté</t>
+          <t>Vu</t>
         </is>
       </c>
       <c r="E12" s="7" t="n"/>
       <c r="F12" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=SJ-43514</t>
+          <t>https://www.mouser.fr/fr/new/alps-alpine/alps-alpine-skrw-tact-switches/</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Prise jack 3,5 mm, CMS</t>
+          <t>Poussoir SKRW — variantes 50k / 500k / 1000k cycles</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>SJ-43514-SMT-TR</t>
+          <t>SKRWAEE030 · SKRWAME030 · SKRWADE030</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Same Sky (CUI Devices)</t>
+          <t>Alps Alpine</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Documenté</t>
+          <t>À confirmer</t>
         </is>
       </c>
       <c r="E13" s="7" t="n"/>
       <c r="F13" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=SJ-43514-SMT-TR</t>
+          <t>https://www.mouser.fr/c/?q=SKRW</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>Micro-USB B, CMS coudée</t>
+          <t>Fusible réarmable PPTC, boîtier 1812</t>
         </is>
       </c>
       <c r="B14" s="10" t="inlineStr">
         <is>
-          <t>10118193-0001LF</t>
+          <t>série MF-MSMF</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Amphenol FCI</t>
+          <t>Bourns</t>
         </is>
       </c>
       <c r="D14" s="11" t="inlineStr">
         <is>
-          <t>Documenté</t>
+          <t>À confirmer</t>
         </is>
       </c>
       <c r="E14" s="7" t="n"/>
       <c r="F14" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=10118193-0001LF</t>
+          <t>https://www.mouser.fr/c/?q=MF-MSMF</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Micro-USB B, variante de montage</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>10118192-0001LF</t>
+          <t>Fusibles PPTC — catalogue complet</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Amphenol FCI</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Variante</t>
+          <t>Catalogue</t>
         </is>
       </c>
       <c r="E15" s="7" t="n"/>
       <c r="F15" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=10118192-0001LF</t>
+          <t>https://www.mouser.fr/c/?q=fusible+PPTC+1812</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>Micro-USB B, variante de montage</t>
-        </is>
-      </c>
-      <c r="B16" s="10" t="inlineStr">
-        <is>
-          <t>10118194-0001LF</t>
+          <t>Haut-parleurs — catalogue</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>Amphenol FCI</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Variante</t>
+          <t>Catalogue</t>
         </is>
       </c>
       <c r="E16" s="7" t="n"/>
       <c r="F16" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=10118194-0001LF</t>
+          <t>https://www.mouser.fr/c/?q=haut-parleur+15mm+8+ohm</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Mini-USB B, 5 contacts</t>
+          <t>Antenne UHF hélicoïdale CMS</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>54819-0519</t>
+          <t>ANT-868-VHETH</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>Molex</t>
+          <t>TE / Linx</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>À confirmer</t>
+          <t>Documenté</t>
         </is>
       </c>
       <c r="E17" s="7" t="n"/>
       <c r="F17" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=54819-0519</t>
+          <t>https://www.mouser.fr/c/?q=ANT-868-VHETH</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>USB-C, 16 contacts, traversante</t>
-        </is>
-      </c>
-      <c r="B18" s="10" t="inlineStr">
-        <is>
-          <t>USB4085-GF-A</t>
+          <t>Antennes 868 MHz — catalogue</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>GCT</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D18" s="11" t="inlineStr">
         <is>
-          <t>À confirmer</t>
+          <t>Catalogue</t>
         </is>
       </c>
       <c r="E18" s="7" t="n"/>
       <c r="F18" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=USB4085-GF-A</t>
+          <t>https://www.mouser.fr/c/?q=antenne+868+MHz</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>Fusible réarmable PPTC, boîtier 1812</t>
+          <t>Batterie lithium plate (LiPo) — remplace les accus Ni-MH</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>série MF-MSMF</t>
+          <t>à relever sur la cellule</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Bourns</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>À confirmer</t>
+          <t>Photo ext.</t>
         </is>
       </c>
       <c r="E19" s="7" t="n"/>
       <c r="F19" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=MF-MSMF</t>
+          <t>https://www.mouser.fr/c/?q=3.7V+Lipo+Battery</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>Fusibles PPTC — catalogue complet</t>
-        </is>
-      </c>
-      <c r="B20" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
+          <t>Inductance blindée 4,7 µH, 4×4 mm (étage boost)</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>SRN4018-4R7M</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Bourns</t>
         </is>
       </c>
       <c r="D20" s="11" t="inlineStr">
         <is>
-          <t>Catalogue</t>
+          <t>Vu</t>
         </is>
       </c>
       <c r="E20" s="7" t="n"/>
       <c r="F20" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=fusible+PPTC+1812</t>
+          <t>https://www.mouser.fr/c/?q=SRN4018-4R7M</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Haut-parleur Ø15 mm, 8 Ω</t>
+          <t>Condensateurs MLCC CMS — catalogue</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>AS01508MR-6-R</t>
+          <t>0603 / 0805 / 1206</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>PUI Audio</t>
+          <t>Murata, Yageo, KEMET</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>À confirmer</t>
+          <t>Vu</t>
         </is>
       </c>
       <c r="E21" s="7" t="n"/>
       <c r="F21" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=AS01508MR-6-R</t>
+          <t>https://www.mouser.fr/c/?q=MLCC+0805</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>Haut-parleurs — catalogue</t>
+          <t>Kits de résistances CMS</t>
         </is>
       </c>
       <c r="B22" s="11" t="inlineStr">
@@ -1081,404 +1081,40 @@
       <c r="E22" s="7" t="n"/>
       <c r="F22" s="12" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=haut-parleur+15mm+8+ohm</t>
+          <t>https://www.mouser.fr/c/?q=resistor+kit+0805</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Poussoir tactile CMS bas profil — série SKRW (corrigé par l'utilisateur)</t>
+          <t>MCU TI MSP430FR2xxx — famille</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>série SKRW</t>
+          <t>réf. exacte à relire sur la puce</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Alps Alpine</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Vu</t>
+          <t>À confirmer</t>
         </is>
       </c>
       <c r="E23" s="7" t="n"/>
       <c r="F23" s="8" t="inlineStr">
         <is>
-          <t>https://www.mouser.fr/c/?q=SKRW</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="9" t="inlineStr">
-        <is>
-          <t>Poussoir tactile SKRW — variantes de durée de vie 50k / 500k / 1000k</t>
-        </is>
-      </c>
-      <c r="B24" s="10" t="inlineStr">
-        <is>
-          <t>SKRWAEE030 · SKRWAME030 · SKRWADE030</t>
-        </is>
-      </c>
-      <c r="C24" s="11" t="inlineStr">
-        <is>
-          <t>Alps Alpine</t>
-        </is>
-      </c>
-      <c r="D24" s="11" t="inlineStr">
-        <is>
-          <t>À confirmer</t>
-        </is>
-      </c>
-      <c r="E24" s="7" t="n"/>
-      <c r="F24" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=SKRWAEE030</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>Bouton poussoir traversant 6 × 6 mm</t>
-        </is>
-      </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>B3F-1000</t>
-        </is>
-      </c>
-      <c r="C25" s="6" t="inlineStr">
-        <is>
-          <t>Omron</t>
-        </is>
-      </c>
-      <c r="D25" s="6" t="inlineStr">
-        <is>
-          <t>À confirmer</t>
-        </is>
-      </c>
-      <c r="E25" s="7" t="n"/>
-      <c r="F25" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=B3F-1000</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="9" t="inlineStr">
-        <is>
-          <t>Antenne UHF hélicoïdale CMS</t>
-        </is>
-      </c>
-      <c r="B26" s="10" t="inlineStr">
-        <is>
-          <t>ANT-868-VHETH</t>
-        </is>
-      </c>
-      <c r="C26" s="11" t="inlineStr">
-        <is>
-          <t>TE / Linx</t>
-        </is>
-      </c>
-      <c r="D26" s="11" t="inlineStr">
-        <is>
-          <t>Documenté</t>
-        </is>
-      </c>
-      <c r="E26" s="7" t="n"/>
-      <c r="F26" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=ANT-868-VHETH</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>Antenne UHF monopole embarqué Ø7 mm</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr">
-        <is>
-          <t>ANT-868-JJB-ST</t>
-        </is>
-      </c>
-      <c r="C27" s="6" t="inlineStr">
-        <is>
-          <t>TE / Linx</t>
-        </is>
-      </c>
-      <c r="D27" s="6" t="inlineStr">
-        <is>
-          <t>Documenté</t>
-        </is>
-      </c>
-      <c r="E27" s="7" t="n"/>
-      <c r="F27" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=ANT-868-JJB-ST</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="9" t="inlineStr">
-        <is>
-          <t>Antenne UHF planaire CMS</t>
-        </is>
-      </c>
-      <c r="B28" s="10" t="inlineStr">
-        <is>
-          <t>ANT-868-SP</t>
-        </is>
-      </c>
-      <c r="C28" s="11" t="inlineStr">
-        <is>
-          <t>TE / Linx</t>
-        </is>
-      </c>
-      <c r="D28" s="11" t="inlineStr">
-        <is>
-          <t>Documenté</t>
-        </is>
-      </c>
-      <c r="E28" s="7" t="n"/>
-      <c r="F28" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=ANT-868-SP</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>Antennes 868 MHz — catalogue</t>
-        </is>
-      </c>
-      <c r="B29" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C29" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D29" s="6" t="inlineStr">
-        <is>
-          <t>Catalogue</t>
-        </is>
-      </c>
-      <c r="E29" s="7" t="n"/>
-      <c r="F29" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=antenne+868+MHz</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="9" t="inlineStr">
-        <is>
-          <t>Inductance blindée 4,7 µH, 4×4 mm (étage boost)</t>
-        </is>
-      </c>
-      <c r="B30" s="10" t="inlineStr">
-        <is>
-          <t>SRN4018-4R7M</t>
-        </is>
-      </c>
-      <c r="C30" s="11" t="inlineStr">
-        <is>
-          <t>Bourns</t>
-        </is>
-      </c>
-      <c r="D30" s="11" t="inlineStr">
-        <is>
-          <t>Vu</t>
-        </is>
-      </c>
-      <c r="E30" s="7" t="n"/>
-      <c r="F30" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=SRN4018-4R7M</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>Condensateurs MLCC CMS — catalogue</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>0603 / 0805 / 1206</t>
-        </is>
-      </c>
-      <c r="C31" s="6" t="inlineStr">
-        <is>
-          <t>Murata, Yageo, KEMET</t>
-        </is>
-      </c>
-      <c r="D31" s="6" t="inlineStr">
-        <is>
-          <t>Vu</t>
-        </is>
-      </c>
-      <c r="E31" s="7" t="n"/>
-      <c r="F31" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=MLCC+0805</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="9" t="inlineStr">
-        <is>
-          <t>Kits de condensateurs</t>
-        </is>
-      </c>
-      <c r="B32" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C32" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D32" s="11" t="inlineStr">
-        <is>
-          <t>Catalogue</t>
-        </is>
-      </c>
-      <c r="E32" s="7" t="n"/>
-      <c r="F32" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=capacitor+kit</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="4" t="inlineStr">
-        <is>
-          <t>Résistances CMS — catalogue</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>RC0805 / CRCW0805</t>
-        </is>
-      </c>
-      <c r="C33" s="6" t="inlineStr">
-        <is>
-          <t>Yageo, Vishay</t>
-        </is>
-      </c>
-      <c r="D33" s="6" t="inlineStr">
-        <is>
-          <t>Vu</t>
-        </is>
-      </c>
-      <c r="E33" s="7" t="n"/>
-      <c r="F33" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=RC0805+resistance</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="9" t="inlineStr">
-        <is>
-          <t>Kits de résistances CMS</t>
-        </is>
-      </c>
-      <c r="B34" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="C34" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D34" s="11" t="inlineStr">
-        <is>
-          <t>Catalogue</t>
-        </is>
-      </c>
-      <c r="E34" s="7" t="n"/>
-      <c r="F34" s="12" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=resistor+kit+0805</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>Batterie lithium plate (LiPo) — remplace les accus AA Ni-MH</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="inlineStr">
-        <is>
-          <t>à relever sur la cellule</t>
-        </is>
-      </c>
-      <c r="C35" s="6" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D35" s="6" t="inlineStr">
-        <is>
-          <t>Photo ext.</t>
-        </is>
-      </c>
-      <c r="E35" s="7" t="n"/>
-      <c r="F35" s="8" t="inlineStr">
-        <is>
-          <t>https://www.mouser.fr/c/?q=batterie+lithium+polymere+3.7V</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="9" t="inlineStr">
-        <is>
-          <t>MCU TI MSP430FR2xxx — famille</t>
-        </is>
-      </c>
-      <c r="B36" s="10" t="inlineStr">
-        <is>
-          <t>réf. exacte à relire sur la puce</t>
-        </is>
-      </c>
-      <c r="C36" s="11" t="inlineStr">
-        <is>
-          <t>Texas Instruments</t>
-        </is>
-      </c>
-      <c r="D36" s="11" t="inlineStr">
-        <is>
-          <t>À confirmer</t>
-        </is>
-      </c>
-      <c r="E36" s="7" t="n"/>
-      <c r="F36" s="12" t="inlineStr">
-        <is>
           <t>https://www.mouser.fr/c/?q=MSP430FR2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:F36"/>
+  <autoFilter ref="A4:F23"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -1503,19 +1139,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId17"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F22" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F23" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F24" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F25" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F26" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F27" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F28" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F29" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F30" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F31" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F32" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId32"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add a tourGuide AIR sheet scoping the list to the affected product
The fault touches one product, but the list still covered seven. A new
sheet keeps only what is seen or attested on the AIR board itself — the
lithium cell, micro-USB charge port, SKRW switches, boost inductor,
0603/0805 passives, headphone jack, the custom segment LCD, and the
charging case inlet — and names, for each line, why it is there.

A second table lists what was deliberately left out and why, since that
is where the earlier lists went wrong: USB-C and the FPC belong to the
Eco 2.0 board, the catalogue antennas do not apply to a device whose
antenna is a spring soldered to the PCB, and the speaker, PPTC fuse and
mini-USB were never observed on this board at all.

The user-settled main sheet is untouched.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ge7EoEedmTKdVGHi238WWF
</commit_message>
<xml_diff>
--- a/exports/Liste-Mouser-Tonwelt-TG288.xlsx
+++ b/exports/Liste-Mouser-Tonwelt-TG288.xlsx
@@ -11,6 +11,7 @@
     <sheet name="Hors Mouser" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Mesures restantes" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Sources &amp; statuts" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="tourGuide AIR" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Liste Mouser'!$A$4:$F$26</definedName>
@@ -22,7 +23,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,6 +63,12 @@
       <color rgb="000563C1"/>
       <sz val="9"/>
       <u val="single"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00E65100"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="5">
@@ -113,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -159,6 +166,13 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1784,4 +1798,414 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="56" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>tourGuide AIR — le seul produit touché par la panne de surchauffe</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Sous-ensemble de la feuille « Liste Mouser », restreint à ce qui est constaté ou attesté sur la carte du tourGuide AIR (les 15 photos macro de diagnostics/talkie-surchauffe/). La feuille principale reste inchangée.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Composant</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Référence</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Statut</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Pourquoi cette ligne</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Lien Mouser</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Cellule lithium plate</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>JHY632570 · 3,7 V · 1300 mAh</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Vu</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Carte à ressort d'antenne + micro-USB — ⚠ reste à confirmer que cette carte est bien l'AIR</t>
+        </is>
+      </c>
+      <c r="E5" s="17" t="inlineStr">
+        <is>
+          <t>https://www.mouser.fr/c/?q=3.7V+Lipo+Battery</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="9" t="inlineStr">
+        <is>
+          <t>Port de charge micro-USB B</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>10118193-0001LF (+ variantes …192 / …194)</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>Documenté</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>Le diagnostic cite le port micro-USB (§6.7, corrosion fréquente en location)</t>
+        </is>
+      </c>
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>https://www.mouser.fr/c/?q=10118193-0001LF</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Poussoirs tactiles CMS</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>série SKRW</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Vu</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Corrigé par l'utilisateur. Suffixe selon durée de vie visée</t>
+        </is>
+      </c>
+      <c r="E7" s="17" t="inlineStr">
+        <is>
+          <t>https://www.mouser.fr/c/?q=SKRW</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="9" t="inlineStr">
+        <is>
+          <t>Inductance blindée 4,7 µH, 4×4 mm</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>SRN4018-4R7M</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>Vu</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>Deux étages à découpage sur la carte</t>
+        </is>
+      </c>
+      <c r="E8" s="18" t="inlineStr">
+        <is>
+          <t>https://www.mouser.fr/c/?q=SRN4018-4R7M</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Condensateurs MLCC 0603 / 0805</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>à relever</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Vu</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>473 = 47 nF identifié sur l'étage boost</t>
+        </is>
+      </c>
+      <c r="E9" s="17" t="inlineStr">
+        <is>
+          <t>https://www.mouser.fr/c/?q=MLCC+0805</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>Résistances 0805</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>à relever</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>Vu</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>3R3 = 3,3 Ω identifié</t>
+        </is>
+      </c>
+      <c r="E10" s="18" t="inlineStr">
+        <is>
+          <t>https://www.mouser.fr/c/?q=RC0805</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Prise jack 3,5 mm (sortie casque)</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>SJ-43514-SMT-TR</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Documenté</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Fiche Linkx : sortie casque sur la version récepteur</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="inlineStr">
+        <is>
+          <t>https://www.mouser.fr/c/?q=SJ-43514-SMT-TR</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="9" t="inlineStr">
+        <is>
+          <t>Écran LCD à segments</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>SUR MESURE — hors catalogue</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>Vu</t>
+        </is>
+      </c>
+      <c r="D12" s="9" t="inlineStr">
+        <is>
+          <t>Pictogrammes propres au produit. SAV Linkx/Tonwelt ou refabrication sur plan</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
+          <t>Prise d'alimentation de la VALISE de charge</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>KPJX-4S-S</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Photo ext.</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Appartient à la valise, pas à l'appareil — mais la valise est suspecte n°4</t>
+        </is>
+      </c>
+      <c r="E13" s="17" t="inlineStr">
+        <is>
+          <t>https://www.mouser.fr/c/?q=KPJX-4S-S</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>Volontairement EXCLU du périmètre AIR</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Écarté</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Pourquoi</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
+        <is>
+          <t>USB-C et nappe FPC</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Ce sont les connecteurs de la carte « Eco 2.0 » (supraGuide ECO), pas de l'AIR</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>Antennes Linx ANT-868-*</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="inlineStr">
+        <is>
+          <t>L'AIR porte un ressort d'antenne soudé sur la carte, pas une antenne de catalogue</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>Prise mini-USB</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Gardée par l'utilisateur, mais non constatée sur la carte de l'AIR — appartient à un autre produit</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>Haut-parleur</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>Non constaté sur l'AIR : c'est un récepteur à écouteurs</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>Fusible PPTC</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Non constaté sur les photos de l'AIR</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="14" t="inlineStr">
+        <is>
+          <t>MCU, SoC RF, driver LCD, TCXO, 4 codes CMS non résolus</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="inlineStr">
+        <is>
+          <t>Voir la feuille « Hors Mouser » : non commandables ou non identifiés</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId8"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>